<commit_message>
Update: Sync latest registrations, fix sports gender classifications, update cover date to 30 Aug 2569 and sync web public assets
</commit_message>
<xml_diff>
--- a/เอกสารและรายชื่อคณะสีแสด_ปี69/แยกฝ่าย/สตาฟ/รายชื่อคณะกรรมการและสตาฟ_คณะสีแสด_ปี69.xlsx
+++ b/เอกสารและรายชื่อคณะสีแสด_ปี69/แยกฝ่าย/สตาฟ/รายชื่อคณะกรรมการและสตาฟ_คณะสีแสด_ปี69.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="280">
   <si>
     <t>👑 รายชื่อคณะกรรมการและทีมงานสตาฟ — คณะสีแสด (สีบุษราคัม) ปี 2569</t>
   </si>
@@ -262,99 +262,102 @@
     <t>นางสาวเกศศิริประภา ใจมา</t>
   </si>
   <si>
+    <t>สตาฟสวัสดิการ, คัลเลอร์การ์ด</t>
+  </si>
+  <si>
+    <t>081-160-6764</t>
+  </si>
+  <si>
+    <t>34759</t>
+  </si>
+  <si>
+    <t>นายณัฐทวัฒน์ เอี้ยงหมี</t>
+  </si>
+  <si>
+    <t>ตะกร้อ</t>
+  </si>
+  <si>
+    <t>099-405-2582</t>
+  </si>
+  <si>
+    <t>ม.5/4</t>
+  </si>
+  <si>
+    <t>32449</t>
+  </si>
+  <si>
+    <t>นายอธิภู คำฟอง</t>
+  </si>
+  <si>
+    <t>สตาฟบาสเกตบอล</t>
+  </si>
+  <si>
+    <t>097-287-1024</t>
+  </si>
+  <si>
+    <t>32510</t>
+  </si>
+  <si>
+    <t>นางสาวศุภิสรา ตาแสงวงษ์</t>
+  </si>
+  <si>
+    <t>ฟุตบอล, ดรัมเมเยอร์</t>
+  </si>
+  <si>
+    <t>061-553-0691</t>
+  </si>
+  <si>
+    <t>32631</t>
+  </si>
+  <si>
+    <t>นางสาวสาริกา ปราณนคร</t>
+  </si>
+  <si>
+    <t>080-887-7109</t>
+  </si>
+  <si>
+    <t>32646</t>
+  </si>
+  <si>
+    <t>นายศักดิธัช จินตา</t>
+  </si>
+  <si>
+    <t>095-935-5206</t>
+  </si>
+  <si>
+    <t>32757</t>
+  </si>
+  <si>
+    <t>นางสาวกานต์พิชชา พฤกษาพรรพต</t>
+  </si>
+  <si>
+    <t>ฟุตบอล, สตาฟฟุตบอลชาย</t>
+  </si>
+  <si>
+    <t>084-989-0044</t>
+  </si>
+  <si>
+    <t>34770</t>
+  </si>
+  <si>
+    <t>นายธนวัฒน์ อุดจอม</t>
+  </si>
+  <si>
+    <t>มือกลอง</t>
+  </si>
+  <si>
+    <t>063-113-6053</t>
+  </si>
+  <si>
+    <t>34776</t>
+  </si>
+  <si>
+    <t>นางสาววิภาดา แก้วตา</t>
+  </si>
+  <si>
     <t>สตาฟสวัสดิการ</t>
   </si>
   <si>
-    <t>081-160-6764</t>
-  </si>
-  <si>
-    <t>34759</t>
-  </si>
-  <si>
-    <t>นายณัฐทวัฒน์ เอี้ยงหมี</t>
-  </si>
-  <si>
-    <t>ตะกร้อ</t>
-  </si>
-  <si>
-    <t>099-405-2582</t>
-  </si>
-  <si>
-    <t>ม.5/4</t>
-  </si>
-  <si>
-    <t>32449</t>
-  </si>
-  <si>
-    <t>นายอธิภู คำฟอง</t>
-  </si>
-  <si>
-    <t>สตาฟบาสเกตบอล</t>
-  </si>
-  <si>
-    <t>097-287-1024</t>
-  </si>
-  <si>
-    <t>32510</t>
-  </si>
-  <si>
-    <t>นางสาวศุภิสรา ตาแสงวงษ์</t>
-  </si>
-  <si>
-    <t>ฟุตบอล, ดรัมเมเยอร์</t>
-  </si>
-  <si>
-    <t>061-553-0691</t>
-  </si>
-  <si>
-    <t>32631</t>
-  </si>
-  <si>
-    <t>นางสาวสาริกา ปราณนคร</t>
-  </si>
-  <si>
-    <t>080-887-7109</t>
-  </si>
-  <si>
-    <t>32646</t>
-  </si>
-  <si>
-    <t>นายศักดิธัช จินตา</t>
-  </si>
-  <si>
-    <t>095-935-5206</t>
-  </si>
-  <si>
-    <t>32757</t>
-  </si>
-  <si>
-    <t>นางสาวกานต์พิชชา พฤกษาพรรพต</t>
-  </si>
-  <si>
-    <t>ฟุตบอล, สตาฟฟุตบอลชาย</t>
-  </si>
-  <si>
-    <t>084-989-0044</t>
-  </si>
-  <si>
-    <t>34770</t>
-  </si>
-  <si>
-    <t>นายธนวัฒน์ อุดจอม</t>
-  </si>
-  <si>
-    <t>มือกลอง</t>
-  </si>
-  <si>
-    <t>063-113-6053</t>
-  </si>
-  <si>
-    <t>34776</t>
-  </si>
-  <si>
-    <t>นางสาววิภาดา แก้วตา</t>
-  </si>
-  <si>
     <t>099-237-8944</t>
   </si>
   <si>
@@ -772,6 +775,12 @@
     <t>นายอิธิกุล โมเฮด</t>
   </si>
   <si>
+    <t>ฝ่ายสวัสดิการ</t>
+  </si>
+  <si>
+    <t>065-496-0745</t>
+  </si>
+  <si>
     <t>32795</t>
   </si>
   <si>
@@ -785,6 +794,9 @@
   </si>
   <si>
     <t>นายพีรพล ทวีทรัพย์ล้ำเลิศ</t>
+  </si>
+  <si>
+    <t>รองประธานคณะสีแสด, กรีฑา, เปตอง, ตะกร้อ, วอลเลย์บอล, บาสเกตบอล, ฟุตบอล, วิ่ง 16 ขา</t>
   </si>
   <si>
     <t>061-267-2452</t>
@@ -2091,10 +2103,10 @@
         <v>13</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="31" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2108,19 +2120,19 @@
         <v>44</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F31" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="32" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2128,16 +2140,16 @@
         <v>29</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C32" s="4">
         <v>23</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>13</v>
@@ -2146,7 +2158,7 @@
         <v>39</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="33" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2154,25 +2166,25 @@
         <v>30</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C33" s="7">
         <v>29</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F33" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="34" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2180,16 +2192,16 @@
         <v>31</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C34" s="4">
         <v>35</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>13</v>
@@ -2206,16 +2218,16 @@
         <v>32</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C35" s="7">
         <v>14</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F35" s="7" t="s">
         <v>18</v>
@@ -2224,7 +2236,7 @@
         <v>39</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="36" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2232,16 +2244,16 @@
         <v>33</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C36" s="4">
         <v>16</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>18</v>
@@ -2250,7 +2262,7 @@
         <v>39</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="37" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2258,25 +2270,25 @@
         <v>34</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C37" s="7">
         <v>41</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F37" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="38" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2284,16 +2296,16 @@
         <v>35</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C38" s="4">
         <v>14</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>13</v>
@@ -2302,7 +2314,7 @@
         <v>44</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="39" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2310,16 +2322,16 @@
         <v>36</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C39" s="7">
         <v>2</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F39" s="7" t="s">
         <v>18</v>
@@ -2328,7 +2340,7 @@
         <v>19</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="40" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2336,25 +2348,25 @@
         <v>37</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C40" s="4">
         <v>20</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="41" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2362,25 +2374,25 @@
         <v>38</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C41" s="7">
         <v>25</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F41" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="42" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2388,25 +2400,25 @@
         <v>39</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C42" s="4">
         <v>7</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>18</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="43" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2414,16 +2426,16 @@
         <v>40</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C43" s="7">
         <v>31</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>13</v>
@@ -2432,7 +2444,7 @@
         <v>110</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="44" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2440,25 +2452,25 @@
         <v>41</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C44" s="4">
         <v>37</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F44" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="45" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2466,16 +2478,16 @@
         <v>42</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C45" s="7">
         <v>4</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F45" s="7" t="s">
         <v>18</v>
@@ -2492,25 +2504,25 @@
         <v>43</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C46" s="4">
         <v>16</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F46" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="47" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2518,16 +2530,16 @@
         <v>44</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C47" s="7">
         <v>5</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F47" s="7" t="s">
         <v>18</v>
@@ -2544,16 +2556,16 @@
         <v>45</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C48" s="4">
         <v>22</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F48" s="4" t="s">
         <v>13</v>
@@ -2562,7 +2574,7 @@
         <v>51</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="49" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2570,16 +2582,16 @@
         <v>46</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C49" s="7">
         <v>27</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F49" s="7" t="s">
         <v>13</v>
@@ -2596,16 +2608,16 @@
         <v>47</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C50" s="4">
         <v>33</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F50" s="4" t="s">
         <v>13</v>
@@ -2614,7 +2626,7 @@
         <v>51</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="51" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2622,25 +2634,25 @@
         <v>48</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C51" s="7">
         <v>17</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F51" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="52" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2648,22 +2660,22 @@
         <v>49</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C52" s="4">
         <v>23</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F52" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H52" s="4" t="s">
         <v>15</v>
@@ -2674,25 +2686,25 @@
         <v>50</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C53" s="7">
         <v>6</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F53" s="7" t="s">
         <v>18</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="54" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2700,16 +2712,16 @@
         <v>51</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C54" s="4">
         <v>29</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F54" s="4" t="s">
         <v>13</v>
@@ -2718,7 +2730,7 @@
         <v>76</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="55" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2726,16 +2738,16 @@
         <v>52</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C55" s="7">
         <v>11</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F55" s="7" t="s">
         <v>18</v>
@@ -2744,7 +2756,7 @@
         <v>51</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="56" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2752,25 +2764,25 @@
         <v>53</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C56" s="4">
         <v>35</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F56" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="57" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2778,16 +2790,16 @@
         <v>54</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C57" s="7">
         <v>13</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F57" s="7" t="s">
         <v>13</v>
@@ -2796,7 +2808,7 @@
         <v>44</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="58" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2804,22 +2816,22 @@
         <v>55</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C58" s="4">
         <v>6</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F58" s="4" t="s">
         <v>18</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H58" s="4" t="s">
         <v>15</v>
@@ -2830,25 +2842,25 @@
         <v>56</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C59" s="7">
         <v>19</v>
       </c>
       <c r="D59" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="E59" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="F59" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G59" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="E59" s="8" t="s">
-        <v>205</v>
-      </c>
-      <c r="F59" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G59" s="9" t="s">
-        <v>203</v>
-      </c>
       <c r="H59" s="7" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="60" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2856,16 +2868,16 @@
         <v>57</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C60" s="4">
         <v>25</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F60" s="4" t="s">
         <v>13</v>
@@ -2874,7 +2886,7 @@
         <v>44</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="61" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2882,16 +2894,16 @@
         <v>58</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C61" s="7">
         <v>2</v>
       </c>
       <c r="D61" s="7" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F61" s="7" t="s">
         <v>18</v>
@@ -2900,7 +2912,7 @@
         <v>92</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="62" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2908,25 +2920,25 @@
         <v>59</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C62" s="4">
         <v>19</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F62" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="63" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2934,25 +2946,25 @@
         <v>60</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C63" s="7">
         <v>7</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F63" s="7" t="s">
         <v>18</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="64" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2960,25 +2972,25 @@
         <v>61</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C64" s="4">
         <v>25</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F64" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="65" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2986,25 +2998,25 @@
         <v>62</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C65" s="7">
         <v>13</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F65" s="7" t="s">
         <v>18</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="66" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3012,25 +3024,25 @@
         <v>63</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C66" s="4">
         <v>2</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F66" s="4" t="s">
         <v>18</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="67" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3038,16 +3050,16 @@
         <v>64</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C67" s="7">
         <v>8</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F67" s="7" t="s">
         <v>18</v>
@@ -3056,7 +3068,7 @@
         <v>92</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="68" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3064,25 +3076,25 @@
         <v>65</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C68" s="4">
         <v>21</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F68" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="H68" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="69" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3090,16 +3102,16 @@
         <v>66</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C69" s="7">
         <v>27</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F69" s="7" t="s">
         <v>13</v>
@@ -3108,7 +3120,7 @@
         <v>14</v>
       </c>
       <c r="H69" s="7" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="70" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3116,16 +3128,16 @@
         <v>67</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C70" s="4">
         <v>14</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F70" s="4" t="s">
         <v>18</v>
@@ -3134,7 +3146,7 @@
         <v>19</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="71" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3142,25 +3154,25 @@
         <v>68</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C71" s="7">
         <v>14</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F71" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G71" s="9" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H71" s="7" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="72" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3168,25 +3180,25 @@
         <v>69</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C72" s="4">
         <v>2</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F72" s="4" t="s">
         <v>18</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>83</v>
+        <v>254</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>15</v>
+        <v>255</v>
       </c>
     </row>
     <row r="73" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3194,16 +3206,16 @@
         <v>70</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C73" s="7">
         <v>20</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="F73" s="7" t="s">
         <v>13</v>
@@ -3212,7 +3224,7 @@
         <v>76</v>
       </c>
       <c r="H73" s="7" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="74" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3220,25 +3232,25 @@
         <v>71</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C74" s="4">
         <v>8</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="F74" s="4" t="s">
         <v>18</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>35</v>
+        <v>261</v>
       </c>
       <c r="H74" s="4" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="75" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3246,16 +3258,16 @@
         <v>72</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C75" s="7">
         <v>26</v>
       </c>
       <c r="D75" s="7" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="F75" s="7" t="s">
         <v>13</v>
@@ -3264,7 +3276,7 @@
         <v>14</v>
       </c>
       <c r="H75" s="7" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="76" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3272,25 +3284,25 @@
         <v>73</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C76" s="4">
         <v>13</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="F76" s="4" t="s">
         <v>13</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="77" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3298,16 +3310,16 @@
         <v>74</v>
       </c>
       <c r="B77" s="7" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C77" s="7">
         <v>2</v>
       </c>
       <c r="D77" s="7" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="E77" s="8" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="F77" s="7" t="s">
         <v>18</v>
@@ -3324,25 +3336,25 @@
         <v>75</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C78" s="4">
         <v>7</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="F78" s="4" t="s">
         <v>18</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="H78" s="4" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
     </row>
     <row r="79" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3350,16 +3362,16 @@
         <v>76</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C79" s="7">
         <v>18</v>
       </c>
       <c r="D79" s="7" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="E79" s="8" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="F79" s="7" t="s">
         <v>13</v>
@@ -3373,22 +3385,22 @@
     </row>
     <row r="80" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="10" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="B80" s="10"/>
       <c r="C80" s="10"/>
       <c r="D80" s="10"/>
       <c r="E80" s="11" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="F80" s="12" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="G80" s="12" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="H80" s="12" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
     </row>
   </sheetData>

</xml_diff>